<commit_message>
importação de ferquile e livintus
</commit_message>
<xml_diff>
--- a/Docs/TABELA FERGUILE_EXPORTAÇÃO_MOVELSUL_2026.xlsx
+++ b/Docs/TABELA FERGUILE_EXPORTAÇÃO_MOVELSUL_2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="EstaPastaDeTrabalho"/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" tabRatio="603"/>
+    <workbookView windowWidth="23040" windowHeight="8400" tabRatio="603"/>
   </bookViews>
   <sheets>
     <sheet name="EXW" sheetId="11" r:id="rId1"/>
@@ -1712,7 +1712,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{3F3E187C-EDD9-499D-B198-08A08E4FBF35}"/>
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{60391B2C-FA52-44C3-9E07-126BF2E77FF5}"/>
   </tableStyles>
   <colors>
     <mruColors>
@@ -12218,11 +12218,11 @@
         <v>18</v>
       </c>
       <c r="N175" s="62">
-        <v>1949</v>
+        <v>2030</v>
       </c>
       <c r="O175" s="47">
         <f>SUM(N175/'BASE DE CÁLCULO'!$B$13)</f>
-        <v>403.51966873706</v>
+        <v>420.289855072464</v>
       </c>
     </row>
     <row r="176" customFormat="1" customHeight="1" spans="1:45">
@@ -12257,11 +12257,11 @@
         <v>19</v>
       </c>
       <c r="N176" s="46">
-        <v>2030</v>
+        <v>1949</v>
       </c>
       <c r="O176" s="47">
         <f>SUM(N176/'BASE DE CÁLCULO'!$B$13)</f>
-        <v>420.289855072464</v>
+        <v>403.51966873706</v>
       </c>
     </row>
     <row r="177" customFormat="1" customHeight="1" spans="1:15">

</xml_diff>